<commit_message>
Added PeopleSoft to the project
</commit_message>
<xml_diff>
--- a/SAP FI/SAP FI Test Data.xlsx
+++ b/SAP FI/SAP FI Test Data.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phil.harris\Documents\UiPath\Demo\SAP FI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phil.harris\Documents\UiPath\Demo\ADO_Integration\SAP FI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAAE567-EB4D-420D-BC0D-D83D9D0FA703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65CF28C-4F59-4D07-86E4-940B61FCAF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57528" yWindow="6192" windowWidth="11520" windowHeight="7308" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45972" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -78,10 +77,10 @@
     <t>USD</t>
   </si>
   <si>
-    <t>Read Google Sheets Data</t>
-  </si>
-  <si>
     <t>UiPath PMW220</t>
+  </si>
+  <si>
+    <t>Read Excel Data</t>
   </si>
 </sst>
 </file>
@@ -408,7 +407,7 @@
     <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <f ca="1">TODAY()</f>
-        <v>45462</v>
+        <v>45575</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>12</v>
@@ -418,16 +417,16 @@
       </c>
       <c r="D2" s="3">
         <f ca="1">TODAY()</f>
-        <v>45462</v>
+        <v>45575</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="H2" s="4">
         <v>40</v>

</xml_diff>